<commit_message>
W03 D1: the Programme Head's introduction deck, markdown and built pptx; Week 1 example rows aligned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124KbFAUFwPsNP9jL1MCV9G
</commit_message>
<xml_diff>
--- a/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
+++ b/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
@@ -636,7 +636,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
   </cols>
@@ -693,7 +693,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L64"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
@@ -1988,7 +1988,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
@@ -2049,7 +2049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>28</v>
       </c>
@@ -2084,7 +2084,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
@@ -2147,7 +2147,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Build 1 logs rebuilt on the US files: the decisions log reconciles sites, claims and remittances
The log builder read its Reconcile rows from clinics, invoices and payments, which the generator
no longer writes, so it stopped on the first missing file. It now lists the ten files as they are
(sites, claims and remittances in place of the three), and the rebuilt decisions log counts each
one's rows from the CSV: 18, 11,356 and 11,343. The challenges log's example entry names the
at-home channel the files now carry, and the two recalc manifests type the new column and
channel names. xlsx_recalc passes on both workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
+++ b/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Nobody in the group had worked in diagnostics, so we could not say what 'home collection' means in the files or who pays for it.</t>
+          <t>Nobody in the group had worked in diagnostics, so we could not say what 'at-home' means in the files or who pays for it.</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Wrote a one-line definition into our vocabulary map and agreed that a home-collection booking is still one booking, counted once.</t>
+          <t>Wrote a one-line definition into our vocabulary map and agreed that an at-home booking is still one booking, counted once.</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">

</xml_diff>

<commit_message>
W03 D1: translation worksheet and both logs to standard v3
The worksheet carries the setting, all five questions in their askers' words and the Weeks 1 and 2
method in one line per move, so it is filled with nothing else open; each part is a question with
who needs the answer and the questions on the way, and the peer check has its own box. Every sheet
title in the challenges and decisions logs is now the question the sheet answers; the layout, the
formulas and the recalc manifests are unchanged and pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5b1faAeRrqkQL3Mis7VGw
</commit_message>
<xml_diff>
--- a/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
+++ b/content/W03/D1/briefs/C2_W03_D01_challenges_log_STUDENT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>How to use this log</t>
+          <t>How do you fill this log?</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Challenges log</t>
+          <t>Where did the group get stuck, and what did it decide?</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Where the group stands</t>
+          <t>How many challenges are still open, and which one goes to the checkpoint?</t>
         </is>
       </c>
     </row>
@@ -2030,14 +2030,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Entry one, as another group might write it</t>
+          <t>What does a good entry one look like?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Copy the shape, not the words. Your entry one is about your own first stop.</t>
+          <t>Another group's entry one. Copy its shape; your entry is about your own first stop.</t>
         </is>
       </c>
     </row>

</xml_diff>